<commit_message>
Remove local image manifest — Supabase Storage is the only image source now
- Delete part_images/ folder and generate-manifest.py
- Remove loadImageManifest() from data.js
- Remove state.localImages from config.js
- Remove localImgs from loadProductImages() in products.js

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NgocThanh_30_12_2026_IN.xlsx
+++ b/NgocThanh_30_12_2026_IN.xlsx
@@ -31,6 +31,14 @@
     </bk>
   </cellMetadata>
 </metadata>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <si>
+    <t>BRE-81045, YNC-123421</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -540,8 +548,8 @@
       <c r="C3" t="str">
         <v>Brembo</v>
       </c>
-      <c r="D3" t="str">
-        <v>BRE-81045</v>
+      <c r="D3" s="0" t="s">
+        <v>0</v>
       </c>
       <c r="E3" t="str">
         <v>Engine</v>

</xml_diff>